<commit_message>
add dsa revision tracker
</commit_message>
<xml_diff>
--- a/DSA_Excel.xlsx
+++ b/DSA_Excel.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrid\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrid\OneDrive\Desktop\DSA\java-data-structures-and-algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F8252F-3410-4E07-AEE5-58DA1992CE17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33939547-2BB8-4121-9900-A6AA4D46B8C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>DSA Problem</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>Approaches</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Easy</t>
   </si>
 </sst>
 </file>
@@ -98,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -109,6 +112,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,6 +432,24 @@
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46322</v>
+      </c>
+      <c r="E2" s="4">
+        <v>46323</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>